<commit_message>
Örnek kur ve endeks verileri
</commit_message>
<xml_diff>
--- a/tcmb_enflasyon_verileri.xlsx
+++ b/tcmb_enflasyon_verileri.xlsx
@@ -20,144 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t xml:space="preserve">Tarih</t>
   </si>
   <si>
     <t xml:space="preserve">Yİ_UFE_Endeks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2021-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2022-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2024-12</t>
   </si>
   <si>
     <t xml:space="preserve">2025-01</t>
@@ -295,7 +163,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -317,6 +185,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -450,8 +322,8 @@
   <dimension ref="A1:B152"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="15.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.7"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -467,7 +339,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>666.79</v>
+        <v>3861.33</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -475,7 +347,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>693.54</v>
+        <v>3943.01</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -483,7 +355,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>710.61</v>
+        <v>4017.3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -491,7 +363,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>730.28</v>
+        <v>4128.19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -499,7 +371,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>741.58</v>
+        <v>4230.69</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -507,7 +379,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>780.45</v>
+        <v>4334.94</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -515,7 +387,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>858.43</v>
+        <v>4409.73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -523,7 +395,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1022.25</v>
+        <v>4518.89</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -531,7 +403,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1129.03</v>
+        <v>4632.89</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -539,7 +411,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1210.6</v>
+        <v>4708.2</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -547,7 +419,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>1321.9</v>
+        <v>4747.63</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -555,7 +427,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>1423.27</v>
+        <v>4783.04</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -563,7 +435,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1548.01</v>
+        <v>4910.53</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -571,7 +443,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1652.75</v>
+        <v>5029.76</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -579,7 +451,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="5" t="n">
-        <v>1738.21</v>
+        <v>5145.36</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -587,633 +459,413 @@
         <v>17</v>
       </c>
       <c r="B17" s="5" t="n">
-        <v>1780.05</v>
+        <v>5308.46</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="5" t="n">
-        <v>1865.09</v>
-      </c>
+      <c r="B18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>2011.13</v>
-      </c>
+      <c r="B19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>2026.08</v>
-      </c>
+      <c r="B20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>2021.19</v>
-      </c>
+      <c r="B21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="5" t="n">
-        <v>2105.17</v>
-      </c>
+      <c r="B22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23" s="5" t="n">
-        <v>2138.04</v>
-      </c>
+      <c r="B23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>2147.44</v>
-      </c>
+      <c r="B24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>2164.94</v>
-      </c>
+      <c r="B25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>2179.02</v>
-      </c>
+      <c r="B26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>2320.72</v>
-      </c>
+      <c r="B27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="B28" s="5" t="n">
-        <v>2511.75</v>
-      </c>
+      <c r="B28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="B29" s="5" t="n">
-        <v>2659.6</v>
-      </c>
+      <c r="B29" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>2749.98</v>
-      </c>
+      <c r="B30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="B31" s="5" t="n">
-        <v>2803.29</v>
-      </c>
+      <c r="B31" s="6"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="B32" s="5" t="n">
-        <v>2882.04</v>
-      </c>
+      <c r="B32" s="6"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="B33" s="5" t="n">
-        <v>2915.02</v>
-      </c>
+      <c r="B33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="B34" s="5" t="n">
-        <v>3035.59</v>
-      </c>
+      <c r="B34" s="6"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>3149.03</v>
-      </c>
+      <c r="B35" s="6"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="B36" s="5" t="n">
-        <v>3252.79</v>
-      </c>
+      <c r="B36" s="6"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="B37" s="5" t="n">
-        <v>3369.98</v>
-      </c>
+      <c r="B37" s="6"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="B38" s="5" t="n">
-        <v>3435.96</v>
-      </c>
+      <c r="B38" s="6"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="B39" s="5" t="n">
-        <v>3483.25</v>
-      </c>
+      <c r="B39" s="6"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="B40" s="5" t="n">
-        <v>3550.88</v>
-      </c>
+      <c r="B40" s="6"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="B41" s="5" t="n">
-        <v>3610.51</v>
-      </c>
+      <c r="B41" s="6"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="B42" s="5" t="n">
-        <v>3659.84</v>
-      </c>
+      <c r="B42" s="6"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="B43" s="5" t="n">
-        <v>3707.1</v>
-      </c>
+      <c r="B43" s="6"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="B44" s="5" t="n">
-        <v>3731.43</v>
-      </c>
+      <c r="B44" s="6"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="B45" s="5" t="n">
-        <v>3746.52</v>
-      </c>
+      <c r="B45" s="6"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="B46" s="5" t="n">
-        <v>3861.33</v>
-      </c>
+      <c r="B46" s="6"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0" t="s">
-        <v>47</v>
-      </c>
-      <c r="B47" s="5" t="n">
-        <v>3943.01</v>
-      </c>
+      <c r="B47" s="6"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="B48" s="5" t="n">
-        <v>4017.3</v>
-      </c>
+      <c r="B48" s="6"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="B49" s="5" t="n">
-        <v>4128.19</v>
-      </c>
+      <c r="B49" s="6"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="B50" s="5" t="n">
-        <v>4230.69</v>
-      </c>
+      <c r="B50" s="6"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="B51" s="5" t="n">
-        <v>4334.94</v>
-      </c>
+      <c r="B51" s="6"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="B52" s="5" t="n">
-        <v>4409.73</v>
-      </c>
+      <c r="B52" s="6"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="B53" s="5" t="n">
-        <v>4518.89</v>
-      </c>
+      <c r="B53" s="6"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="B54" s="5" t="n">
-        <v>4632.89</v>
-      </c>
+      <c r="B54" s="6"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="B55" s="5" t="n">
-        <v>4708.2</v>
-      </c>
+      <c r="B55" s="6"/>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="B56" s="5" t="n">
-        <v>4747.63</v>
-      </c>
+      <c r="B56" s="6"/>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="0" t="s">
-        <v>57</v>
-      </c>
-      <c r="B57" s="5" t="n">
-        <v>4783.04</v>
-      </c>
+      <c r="B57" s="6"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="B58" s="5" t="n">
-        <v>4910.53</v>
-      </c>
+      <c r="B58" s="6"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="B59" s="5" t="n">
-        <v>5029.76</v>
-      </c>
+      <c r="B59" s="6"/>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="B60" s="5" t="n">
-        <v>5145.36</v>
-      </c>
+      <c r="B60" s="6"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="0" t="s">
-        <v>61</v>
-      </c>
-      <c r="B61" s="5" t="n">
-        <v>5308.46</v>
-      </c>
+      <c r="B61" s="6"/>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="6"/>
+      <c r="B62" s="7"/>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="6"/>
+      <c r="B63" s="7"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="6"/>
+      <c r="B64" s="7"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B65" s="6"/>
+      <c r="B65" s="7"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B66" s="6"/>
+      <c r="B66" s="7"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B67" s="6"/>
+      <c r="B67" s="7"/>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B68" s="6"/>
+      <c r="B68" s="7"/>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="6"/>
+      <c r="B69" s="7"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B70" s="6"/>
+      <c r="B70" s="7"/>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B71" s="6"/>
+      <c r="B71" s="7"/>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B72" s="6"/>
+      <c r="B72" s="7"/>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B73" s="6"/>
+      <c r="B73" s="7"/>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B74" s="6"/>
+      <c r="B74" s="7"/>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B75" s="6"/>
+      <c r="B75" s="7"/>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B76" s="6"/>
+      <c r="B76" s="7"/>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B77" s="6"/>
+      <c r="B77" s="7"/>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B78" s="6"/>
+      <c r="B78" s="7"/>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B79" s="6"/>
+      <c r="B79" s="7"/>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B80" s="6"/>
+      <c r="B80" s="7"/>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B81" s="6"/>
+      <c r="B81" s="7"/>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B82" s="6"/>
+      <c r="B82" s="7"/>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B83" s="6"/>
+      <c r="B83" s="7"/>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B84" s="6"/>
+      <c r="B84" s="7"/>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B85" s="6"/>
+      <c r="B85" s="7"/>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B86" s="6"/>
+      <c r="B86" s="7"/>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B87" s="6"/>
+      <c r="B87" s="7"/>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B88" s="6"/>
+      <c r="B88" s="7"/>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B89" s="6"/>
+      <c r="B89" s="7"/>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B90" s="6"/>
+      <c r="B90" s="7"/>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B91" s="6"/>
+      <c r="B91" s="7"/>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B92" s="6"/>
+      <c r="B92" s="7"/>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B93" s="6"/>
+      <c r="B93" s="7"/>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B94" s="6"/>
+      <c r="B94" s="7"/>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B95" s="6"/>
+      <c r="B95" s="7"/>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B96" s="6"/>
+      <c r="B96" s="7"/>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B97" s="6"/>
+      <c r="B97" s="7"/>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B98" s="6"/>
+      <c r="B98" s="7"/>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B99" s="6"/>
+      <c r="B99" s="7"/>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B100" s="6"/>
+      <c r="B100" s="7"/>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B101" s="6"/>
+      <c r="B101" s="7"/>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B102" s="6"/>
+      <c r="B102" s="7"/>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B103" s="6"/>
+      <c r="B103" s="7"/>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B104" s="6"/>
+      <c r="B104" s="7"/>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B105" s="6"/>
+      <c r="B105" s="7"/>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B106" s="6"/>
+      <c r="B106" s="7"/>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B107" s="6"/>
+      <c r="B107" s="7"/>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B108" s="6"/>
+      <c r="B108" s="7"/>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B109" s="6"/>
+      <c r="B109" s="7"/>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B110" s="6"/>
+      <c r="B110" s="7"/>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B111" s="6"/>
+      <c r="B111" s="7"/>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B112" s="6"/>
+      <c r="B112" s="7"/>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B113" s="6"/>
+      <c r="B113" s="7"/>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B114" s="6"/>
+      <c r="B114" s="7"/>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B115" s="6"/>
+      <c r="B115" s="7"/>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B116" s="6"/>
+      <c r="B116" s="7"/>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B117" s="6"/>
+      <c r="B117" s="7"/>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B118" s="6"/>
+      <c r="B118" s="7"/>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B119" s="6"/>
+      <c r="B119" s="7"/>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B120" s="6"/>
+      <c r="B120" s="7"/>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B121" s="6"/>
+      <c r="B121" s="7"/>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B122" s="6"/>
+      <c r="B122" s="7"/>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B123" s="6"/>
+      <c r="B123" s="7"/>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B124" s="6"/>
+      <c r="B124" s="7"/>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B125" s="6"/>
+      <c r="B125" s="7"/>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B126" s="6"/>
+      <c r="B126" s="7"/>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B127" s="6"/>
+      <c r="B127" s="7"/>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B128" s="6"/>
+      <c r="B128" s="7"/>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B129" s="6"/>
+      <c r="B129" s="7"/>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B130" s="6"/>
+      <c r="B130" s="7"/>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B131" s="6"/>
+      <c r="B131" s="7"/>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B132" s="6"/>
+      <c r="B132" s="7"/>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B133" s="6"/>
+      <c r="B133" s="7"/>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B134" s="6"/>
+      <c r="B134" s="7"/>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B135" s="6"/>
+      <c r="B135" s="7"/>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B136" s="6"/>
+      <c r="B136" s="7"/>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B137" s="6"/>
+      <c r="B137" s="7"/>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B138" s="6"/>
+      <c r="B138" s="7"/>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B139" s="6"/>
+      <c r="B139" s="7"/>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B140" s="6"/>
+      <c r="B140" s="7"/>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B141" s="6"/>
+      <c r="B141" s="7"/>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B142" s="6"/>
+      <c r="B142" s="7"/>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B143" s="6"/>
+      <c r="B143" s="7"/>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B144" s="6"/>
+      <c r="B144" s="7"/>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B145" s="6"/>
+      <c r="B145" s="7"/>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B146" s="6"/>
+      <c r="B146" s="7"/>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B147" s="6"/>
+      <c r="B147" s="7"/>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B148" s="6"/>
+      <c r="B148" s="7"/>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B149" s="6"/>
+      <c r="B149" s="7"/>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B150" s="6"/>
+      <c r="B150" s="7"/>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B151" s="6"/>
+      <c r="B151" s="7"/>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B152" s="6"/>
+      <c r="B152" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>